<commit_message>
Restore old taxonomy and append revised tree
</commit_message>
<xml_diff>
--- a/面向多模态模型的攻击方法体系化梳理_2026-08-21_机制分类合并版.xlsx
+++ b/面向多模态模型的攻击方法体系化梳理_2026-08-21_机制分类合并版.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R974b08a8abf84b83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类树" sheetId="2" r:id="Rb1f1f5afc2624db8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="方法库" sheetId="3" r:id="R75fd033c0a3d441a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源清单" sheetId="4" r:id="R9971b2c3ba3f4e73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径与评分" sheetId="5" r:id="R40ab3023d8914cfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Re0d2368a12d6484c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类树" sheetId="2" r:id="R3e3a89fb698b4e51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="方法库" sheetId="3" r:id="R635a9fa01fe44330"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源清单" sheetId="4" r:id="R6d1c44e8e7844892"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径与评分" sheetId="5" r:id="R910d63f19dbf4b36"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -98,9 +98,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">先在“分类树”按攻击原理定位家族</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">越狱</x:t>
@@ -2488,7 +2485,7 @@
     <x:numFmt numFmtId="164" formatCode="General"/>
     <x:numFmt numFmtId="165" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="47">
+  <x:fonts count="53">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -2744,8 +2741,40 @@
       <x:color rgb="FF7F6000"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF607080"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF607080"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF607080"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FFC62828"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF6A3FC8"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="23">
+  <x:fills count="30">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -2857,8 +2886,43 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF173753"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F7FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF128A8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE9E7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F5EF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1E8FF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="12">
+  <x:borders count="13">
     <x:border diagonalUp="0" diagonalDown="0"/>
     <x:border diagonalUp="0" diagonalDown="0">
       <x:left style="thin">
@@ -2936,6 +3000,20 @@
         <x:color rgb="FFD6DEE6"/>
       </x:bottom>
     </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FFE2C66B"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE2C66B"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE2C66B"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE2C66B"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="21">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2966,7 +3044,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="118">
+  <x:cellXfs count="143">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
       <x:alignment horizontal="general" vertical="center" wrapText="0"/>
     </x:xf>
@@ -3320,6 +3398,81 @@
     </x:xf>
     <x:xf numFmtId="164" fontId="46" fillId="13" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="34" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="35" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="47" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="48" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="49" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="34" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="38" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="38" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="38" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="50" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="50" fillId="26" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="51" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="33" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="52" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="7">
@@ -4031,7 +4184,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7a9a6f7be53a4b56"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7a26514555314587"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4041,19 +4194,31 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TaxonomyTable" displayName="TaxonomyTable" ref="A4:E22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TaxonomyOldTable" displayName="TaxonomyOldTable" ref="A4:E24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="一级分类"/>
     <x:tableColumn id="2" name="二级分类（攻击原理）"/>
     <x:tableColumn id="3" name="原理摘要"/>
     <x:tableColumn id="4" name="代表方法"/>
-    <x:tableColumn id="5" name="调整理由"/>
+    <x:tableColumn id="5" name="该行存在的问题"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TaxonomyNewTable" displayName="TaxonomyNewTable" ref="A29:D47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="一级分类"/>
+    <x:tableColumn id="2" name="二级分类（攻击原理）"/>
+    <x:tableColumn id="3" name="原理摘要"/>
+    <x:tableColumn id="4" name="代表方法"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="AttackMethods" displayName="AttackMethods" ref="A4:AL56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="38">
     <x:tableColumn id="1" name="ID"/>
@@ -4099,7 +4264,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SourcesTable" displayName="SourcesTable" ref="A4:I46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:I46"/>
   <x:tableColumns count="9">
@@ -4373,40 +4538,40 @@
       <x:c r="D5" s="8" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="E5" s="9" t="s">
-        <x:v>7</x:v>
+      <x:c r="E5" s="9" t="str">
+        <x:v>先看“分类树”上半部旧表的问题，再使用下方新机制分类树定位家族</x:v>
       </x:c>
       <x:c r="F5" s="9"/>
     </x:row>
     <x:row r="6" ht="17.350000381469727" hidden="0" customHeight="1">
       <x:c r="A6" s="6" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B6" s="7" t="n">
         <x:f aca="0">COUNTIF('方法库'!$B$5:$B$56,"越狱")</x:f>
         <x:v>41</x:v>
       </x:c>
       <x:c r="D6" s="8" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E6" s="9" t="s">
         <x:v>9</x:v>
-      </x:c>
-      <x:c r="E6" s="9" t="s">
-        <x:v>10</x:v>
       </x:c>
       <x:c r="F6" s="9"/>
     </x:row>
     <x:row r="7" ht="17.350000381469727" hidden="0" customHeight="1">
       <x:c r="A7" s="6" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B7" s="7" t="n">
         <x:f aca="0">COUNTIF('方法库'!$B$5:$B$56,"提示注入")</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="D7" s="8" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E7" s="9" t="s">
         <x:v>12</x:v>
-      </x:c>
-      <x:c r="E7" s="9" t="s">
-        <x:v>13</x:v>
       </x:c>
       <x:c r="F7" s="9"/>
     </x:row>
@@ -4419,40 +4584,40 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="8" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E8" s="9" t="s">
         <x:v>14</x:v>
-      </x:c>
-      <x:c r="E8" s="9" t="s">
-        <x:v>15</x:v>
       </x:c>
       <x:c r="F8" s="9"/>
     </x:row>
     <x:row r="9" ht="17.350000381469727" hidden="0" customHeight="1">
       <x:c r="A9" s="10" t="s">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B9" s="11" t="n">
         <x:f aca="0">COUNTIF('方法库'!$W$5:$W$56,"官方开源")+COUNTIF('方法库'!$W$5:$W$56,"官方项目/代码")+COUNTIF('方法库'!$W$5:$W$56,"第三方统一复现")+COUNTIF('方法库'!$W$5:$W$56,"公开代码/数据")+COUNTIF('方法库'!$W$5:$W$56,"官方/披露方公开代码或材料")</x:f>
         <x:v>31</x:v>
       </x:c>
       <x:c r="D9" s="8" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E9" s="9" t="s">
         <x:v>17</x:v>
-      </x:c>
-      <x:c r="E9" s="9" t="s">
-        <x:v>18</x:v>
       </x:c>
       <x:c r="F9" s="9"/>
     </x:row>
     <x:row r="11" ht="14.25" hidden="0">
       <x:c r="A11" s="12" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B11" s="12" t="s">
         <x:v>19</x:v>
-      </x:c>
-      <x:c r="B11" s="12" t="s">
-        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="14.25" hidden="0">
       <x:c r="A12" s="13" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B12" s="13" t="n">
         <x:f aca="0">COUNTIF('方法库'!$B$5:$B$56,A12)</x:f>
@@ -4461,7 +4626,7 @@
     </x:row>
     <x:row r="13" ht="14.25" hidden="0">
       <x:c r="A13" s="13" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B13" s="13" t="n">
         <x:f aca="0">COUNTIF('方法库'!$B$5:$B$56,A13)</x:f>
@@ -4479,7 +4644,7 @@
     </x:row>
     <x:row r="25" ht="14.25" hidden="0" customHeight="1">
       <x:c r="A25" s="14" t="s">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B25" s="14"/>
       <x:c r="C25" s="14"/>
@@ -4528,7 +4693,7 @@
     <x:mergeCell ref="A27:H27"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86100a4afa1d4160"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ffa0bf72895468b"/>
 </x:worksheet>
 </file>
 
@@ -4537,399 +4702,703 @@
   <x:sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="14.25"/>
   <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="36" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="62" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="60" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="49" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="76" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" hidden="0" customHeight="1">
-      <x:c r="A1" s="67" t="str">
-        <x:v>分类树：按模型实际利用的攻击机制组织</x:v>
-      </x:c>
-      <x:c r="B1" s="67"/>
-      <x:c r="C1" s="67"/>
-      <x:c r="D1" s="67"/>
-      <x:c r="E1" s="71"/>
+      <x:c r="A1" s="121" t="str">
+        <x:v>分类树：按攻击原理组织</x:v>
+      </x:c>
+      <x:c r="B1" s="121"/>
+      <x:c r="C1" s="121"/>
+      <x:c r="D1" s="121"/>
+      <x:c r="E1" s="121"/>
     </x:row>
     <x:row r="2" ht="28" hidden="0" customHeight="1">
-      <x:c r="A2" s="73" t="str">
-        <x:v>二级分类不再按载荷外观或应用场景命名；右侧说明本次机制化重分类的理由。</x:v>
-      </x:c>
-      <x:c r="B2" s="73"/>
-      <x:c r="C2" s="73"/>
-      <x:c r="D2" s="73"/>
-      <x:c r="E2" s="73"/>
+      <x:c r="A2" s="125" t="str">
+        <x:v>二级分类强调模型被利用的机制，而非仅按载荷外观分组。</x:v>
+      </x:c>
+      <x:c r="B2" s="125"/>
+      <x:c r="C2" s="125"/>
+      <x:c r="D2" s="125"/>
+      <x:c r="E2" s="125"/>
       <x:c r="F2" s="2"/>
       <x:c r="G2" s="2"/>
       <x:c r="H2" s="2"/>
     </x:row>
     <x:row r="4" ht="34" hidden="0" customHeight="1">
-      <x:c r="A4" s="81" t="str">
+      <x:c r="A4" s="131" t="str">
         <x:v>一级分类</x:v>
       </x:c>
-      <x:c r="B4" s="81" t="str">
+      <x:c r="B4" s="131" t="str">
         <x:v>二级分类（攻击原理）</x:v>
       </x:c>
-      <x:c r="C4" s="81" t="str">
+      <x:c r="C4" s="131" t="str">
         <x:v>原理摘要</x:v>
       </x:c>
-      <x:c r="D4" s="81" t="str">
+      <x:c r="D4" s="131" t="str">
         <x:v>代表方法</x:v>
       </x:c>
-      <x:c r="E4" s="82" t="str">
-        <x:v>调整理由</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="88" hidden="0" customHeight="1">
-      <x:c r="A5" s="92" t="str">
+      <x:c r="E4" s="131" t="str">
+        <x:v>该行存在的问题</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="66" hidden="0" customHeight="1">
+      <x:c r="A5" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B5" s="86" t="str">
+      <x:c r="B5" s="43" t="str">
+        <x:v>视觉排版与跨模态语义载体</x:v>
+      </x:c>
+      <x:c r="C5" s="43" t="str">
+        <x:v>把敏感语义从文本迁移到图像/OCR/相关图像，使文本审核与视觉理解安全性不一致。</x:v>
+      </x:c>
+      <x:c r="D5" s="43" t="str">
+        <x:v>FigStep、QR、HADES</x:v>
+      </x:c>
+      <x:c r="E5" s="136" t="str">
+        <x:v>分类依据偏向载荷外观（排版、OCR、相关图像），没有明确模型利用的是视觉语义迁移；HADES还包含连续优化阶段。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="66" hidden="0" customHeight="1">
+      <x:c r="A6" s="138" t="str">
+        <x:v>越狱</x:v>
+      </x:c>
+      <x:c r="B6" s="43" t="str">
+        <x:v>跨模态语义拆分与重组</x:v>
+      </x:c>
+      <x:c r="C6" s="43" t="str">
+        <x:v>完整意图仅在多模态或多图重构后出现，各局部载荷风险较低。</x:v>
+      </x:c>
+      <x:c r="D6" s="43" t="str">
+        <x:v>MML、HIMRD、CrossTALK、DMN</x:v>
+      </x:c>
+      <x:c r="E6" s="136" t="str">
+        <x:v>“拆分与重组”范围过窄，漏掉语义编码、多图引用和跨模态重构；Visual Object Replacement、SSJ、AdvBench-Omni等新方法难以准确归类。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="66" hidden="0" customHeight="1">
+      <x:c r="A7" s="138" t="str">
+        <x:v>越狱</x:v>
+      </x:c>
+      <x:c r="B7" s="43" t="str">
+        <x:v>视觉混淆、OOD与注意力分散</x:v>
+      </x:c>
+      <x:c r="C7" s="43" t="str">
+        <x:v>通过打乱、OOD化、拼图、流程图等改变输入分布或分散注意力。</x:v>
+      </x:c>
+      <x:c r="D7" s="43" t="str">
+        <x:v>SI-Attack、JOOD、CS-DJ、FC-Attack</x:v>
+      </x:c>
+      <x:c r="E7" s="136" t="str">
+        <x:v>把输入结构/OOD绕过、注意力分散和流程化解题混成一类；SI-Attack/JOOD、CS-DJ、FC-Attack的主机制不同，必须拆分。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="66" hidden="0" customHeight="1">
+      <x:c r="A8" s="138" t="str">
+        <x:v>越狱</x:v>
+      </x:c>
+      <x:c r="B8" s="43" t="str">
+        <x:v>角色扮演、场景与推理链诱导</x:v>
+      </x:c>
+      <x:c r="C8" s="43" t="str">
+        <x:v>利用角色一致性、叙事、游戏目标或视觉推理链与安全目标竞争。</x:v>
+      </x:c>
+      <x:c r="D8" s="43" t="str">
+        <x:v>VRP、VoiceJailbreak、VisCRA、VisCo、GAMBIT</x:v>
+      </x:c>
+      <x:c r="E8" s="136" t="str">
+        <x:v>把角色/情境诱导与结构化解题/推理链诱导混在一起；VRP、VoiceJailbreak、VisCo与FC-Attack、VisCRA、GAMBIT应分开。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="66" hidden="0" customHeight="1">
+      <x:c r="A9" s="138" t="str">
+        <x:v>越狱</x:v>
+      </x:c>
+      <x:c r="B9" s="43" t="str">
+        <x:v>连续空间对抗优化</x:v>
+      </x:c>
+      <x:c r="C9" s="43" t="str">
+        <x:v>利用图像/音频连续空间、视觉编码或融合状态梯度，优化通用或定向越狱载荷。</x:v>
+      </x:c>
+      <x:c r="D9" s="43" t="str">
+        <x:v>Visual AE、Jailbreak in Pieces、imgJP、UMK、BAP、GBJI</x:v>
+      </x:c>
+      <x:c r="E9" s="136" t="str">
+        <x:v>只写“连续空间”不足以覆盖图像、音频与文本的联合优化；JAMA核心是音频与文本联合优化，应从泛音频类移入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="66" hidden="0" customHeight="1">
+      <x:c r="A10" s="138" t="str">
+        <x:v>越狱</x:v>
+      </x:c>
+      <x:c r="B10" s="43" t="str">
+        <x:v>训练、记忆与传播型</x:v>
+      </x:c>
+      <x:c r="C10" s="43" t="str">
+        <x:v>通过训练投毒、代理记忆或通信把越狱行为持久化并扩散。</x:v>
+      </x:c>
+      <x:c r="D10" s="43" t="str">
+        <x:v>ImgTrojan、Agent Smith</x:v>
+      </x:c>
+      <x:c r="E10" s="136" t="str">
+        <x:v>把训练投毒、Agent记忆和多智能体传播混为模型级机制；主表只应保留训练阶段ImgTrojan，Agent Smith属于应用/Agent链路。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="66" hidden="0" customHeight="1">
+      <x:c r="A11" s="138" t="str">
+        <x:v>越狱</x:v>
+      </x:c>
+      <x:c r="B11" s="43" t="str">
+        <x:v>音频语义与声学弱点</x:v>
+      </x:c>
+      <x:c r="C11" s="43" t="str">
+        <x:v>利用语音叙事、语言/口音覆盖不均、声学变换或音文联合优化。</x:v>
+      </x:c>
+      <x:c r="D11" s="43" t="str">
+        <x:v>VoiceJailbreak、Multi-AudioJail、JAMA</x:v>
+      </x:c>
+      <x:c r="E11" s="136" t="str">
+        <x:v>类别过宽，混入叙事情境（VoiceJailbreak）和联合优化（JAMA）；应聚焦音频载荷、韵律/噪声/声学诱导，并纳入SWhisper等。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="66" hidden="0" customHeight="1">
+      <x:c r="A12" s="138" t="str">
+        <x:v>越狱</x:v>
+      </x:c>
+      <x:c r="B12" s="43" t="str">
+        <x:v>系统提示泄露与自动搜索</x:v>
+      </x:c>
+      <x:c r="C12" s="43" t="str">
+        <x:v>先获取防御信息或依据目标反馈自动演化提示。</x:v>
+      </x:c>
+      <x:c r="D12" s="43" t="str">
+        <x:v>SASP、AutoJailbreak</x:v>
+      </x:c>
+      <x:c r="E12" s="136" t="str">
+        <x:v>把“系统提示泄露”误当主机制；SASP和AutoJailbreak的共同核心是自动生成、评分和反馈搜索，系统提示只是SASP的辅助信息。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="66" hidden="0" customHeight="1">
+      <x:c r="A13" s="140" t="str">
+        <x:v>提示注入</x:v>
+      </x:c>
+      <x:c r="B13" s="43" t="str">
+        <x:v>显式视觉/音频载荷</x:v>
+      </x:c>
+      <x:c r="C13" s="43" t="str">
+        <x:v>把人或OCR/ASR可读的命令放入图片、视频帧或声音。</x:v>
+      </x:c>
+      <x:c r="D13" s="43" t="str">
+        <x:v>Visual OCR Injection、Audible/Video-frame Instruction</x:v>
+      </x:c>
+      <x:c r="E13" s="136" t="str">
+        <x:v>主机制基本正确，但“视频帧”超出本次图、文、音频范围；还需强调媒体中的文字/语音被模型错误当成可执行指令。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="66" hidden="0" customHeight="1">
+      <x:c r="A14" s="140" t="str">
+        <x:v>提示注入</x:v>
+      </x:c>
+      <x:c r="B14" s="43" t="str">
+        <x:v>元数据与外部资源间接注入</x:v>
+      </x:c>
+      <x:c r="C14" s="43" t="str">
+        <x:v>通过媒体元数据、网页/邮件/附件等第三方资源进入上下文。</x:v>
+      </x:c>
+      <x:c r="D14" s="43" t="str">
+        <x:v>Media Metadata Injection、Indirect Multimodal Resource Injection</x:v>
+      </x:c>
+      <x:c r="E14" s="136" t="str">
+        <x:v>主要描述元数据、网页、邮件、附件等应用链路，而不是模型收到图文音输入后自身被利用的机制；应移出当前主表。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="66" hidden="0" customHeight="1">
+      <x:c r="A15" s="140" t="str">
+        <x:v>提示注入</x:v>
+      </x:c>
+      <x:c r="B15" s="43" t="str">
+        <x:v>隐式对抗扰动与语义碰撞</x:v>
+      </x:c>
+      <x:c r="C15" s="43" t="str">
+        <x:v>用不可感知扰动、行为匹配或隐藏状态对齐把指令编码进媒体。</x:v>
+      </x:c>
+      <x:c r="D15" s="43" t="str">
+        <x:v>Instruction Blending、Image Hijacks、IPI、AdvPIA、CrossMPI</x:v>
+      </x:c>
+      <x:c r="E15" s="136" t="str">
+        <x:v>把三种机制混在一起：隐蔽呈现/预处理差异、视觉语义编码、连续空间对抗对齐；InkJect/Anamorpher/IPI、NVIDIA Rebus、Instruction Blending等应分列。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="66" hidden="0" customHeight="1">
+      <x:c r="A16" s="140" t="str">
+        <x:v>提示注入</x:v>
+      </x:c>
+      <x:c r="B16" s="43" t="str">
+        <x:v>上下文劫持与持续对话污染</x:v>
+      </x:c>
+      <x:c r="C16" s="43" t="str">
+        <x:v>初始媒体污染会话历史，使后续轮次持续执行攻击者策略。</x:v>
+      </x:c>
+      <x:c r="D16" s="43" t="str">
+        <x:v>Instruction Blending—Dialog Poisoning</x:v>
+      </x:c>
+      <x:c r="E16" s="136" t="str">
+        <x:v>“持续污染”是多轮攻击效果或持久性，不是根攻击机制；Dialog Poisoning仍属于Adversarial Instruction Blending。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="66" hidden="0" customHeight="1">
+      <x:c r="A17" s="140" t="str">
+        <x:v>提示注入</x:v>
+      </x:c>
+      <x:c r="B17" s="43" t="str">
+        <x:v>跨模态代理与工具劫持</x:v>
+      </x:c>
+      <x:c r="C17" s="43" t="str">
+        <x:v>跨模态载荷直接操纵代理决策、工具调用或连续语音工作流。</x:v>
+      </x:c>
+      <x:c r="D17" s="43" t="str">
+        <x:v>CrossInject、Concurrent Audio PI</x:v>
+      </x:c>
+      <x:c r="E17" s="136" t="str">
+        <x:v>主要描述Agent决策与工具调用劫持等应用链路结果，不是模型级图文音攻击机制；应移出当前主表。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="66" hidden="0" customHeight="1">
+      <x:c r="A18" s="142" t="str">
+        <x:v>数据提取</x:v>
+      </x:c>
+      <x:c r="B18" s="43" t="str">
+        <x:v>训练样本记忆复现与近邻筛选</x:v>
+      </x:c>
+      <x:c r="C18" s="43" t="str">
+        <x:v>利用生成模型对重复样本的记忆，通过批量生成与近邻过滤恢复训练图像。</x:v>
+      </x:c>
+      <x:c r="D18" s="43" t="str">
+        <x:v>Extract-DM</x:v>
+      </x:c>
+      <x:c r="E18" s="136" t="str">
+        <x:v>属于训练数据提取/样本恢复目标，不是越狱或提示注入；本版研究范围暂不纳入数据提取。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="66" hidden="0" customHeight="1">
+      <x:c r="A19" s="142" t="str">
+        <x:v>数据提取</x:v>
+      </x:c>
+      <x:c r="B19" s="43" t="str">
+        <x:v>训练集成员关系推断</x:v>
+      </x:c>
+      <x:c r="C19" s="43" t="str">
+        <x:v>利用训练成员与留出样本在去噪误差上的统计差异判断数据是否参与训练。</x:v>
+      </x:c>
+      <x:c r="D19" s="43" t="str">
+        <x:v>SecMI</x:v>
+      </x:c>
+      <x:c r="E19" s="136" t="str">
+        <x:v>属于成员推断的数据隐私攻击，与当前仅保留的越狱/提示注入目标不同；本版暂不纳入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="66" hidden="0" customHeight="1">
+      <x:c r="A20" s="142" t="str">
+        <x:v>数据提取</x:v>
+      </x:c>
+      <x:c r="B20" s="43" t="str">
+        <x:v>跨模态置信度成员推断</x:v>
+      </x:c>
+      <x:c r="C20" s="43" t="str">
+        <x:v>聚合视觉语言模型高信息token的异常置信信号，判断图像、文本或图文对的成员关系。</x:v>
+      </x:c>
+      <x:c r="D20" s="43" t="str">
+        <x:v>VL-MIA</x:v>
+      </x:c>
+      <x:c r="E20" s="136" t="str">
+        <x:v>属于跨模态成员推断/置信度攻击，仍是数据提取方向；本版暂不纳入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="66" hidden="0" customHeight="1">
+      <x:c r="A21" s="142" t="str">
+        <x:v>数据提取</x:v>
+      </x:c>
+      <x:c r="B21" s="43" t="str">
+        <x:v>视频时序记忆成员推断</x:v>
+      </x:c>
+      <x:c r="C21" s="43" t="str">
+        <x:v>利用跨帧顺序与动态依赖产生的记忆差异，在纯黑盒输出下判断视频成员关系。</x:v>
+      </x:c>
+      <x:c r="D21" s="43" t="str">
+        <x:v>VideoMIA</x:v>
+      </x:c>
+      <x:c r="E21" s="136" t="str">
+        <x:v>同时属于视频专属与成员推断方向，超出当前图、文、音频及越狱/提示注入范围。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="66" hidden="0" customHeight="1">
+      <x:c r="A22" s="142" t="str">
+        <x:v>数据提取</x:v>
+      </x:c>
+      <x:c r="B22" s="43" t="str">
+        <x:v>跨模态潜变量反演与成员推断</x:v>
+      </x:c>
+      <x:c r="C22" s="43" t="str">
+        <x:v>用文本引导CLIP/CLAP潜变量反演，从相似度和稳定性推断图像/音频PII成员关系。</x:v>
+      </x:c>
+      <x:c r="D22" s="43" t="str">
+        <x:v>UMID</x:v>
+      </x:c>
+      <x:c r="E22" s="136" t="str">
+        <x:v>属于潜变量反演与成员推断的数据隐私攻击；本版暂不纳入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="66" hidden="0" customHeight="1">
+      <x:c r="A23" s="142" t="str">
+        <x:v>数据提取</x:v>
+      </x:c>
+      <x:c r="B23" s="43" t="str">
+        <x:v>系统提示词直接诱导与多轮复述</x:v>
+      </x:c>
+      <x:c r="C23" s="43" t="str">
+        <x:v>通过多轮改写、局部复述和格式诱导，让模型披露系统提示及隐藏规则。</x:v>
+      </x:c>
+      <x:c r="D23" s="43" t="str">
+        <x:v>GPT-4V SPA</x:v>
+      </x:c>
+      <x:c r="E23" s="136" t="str">
+        <x:v>攻击目标是系统提示/隐藏规则泄露，属于数据提取；不要与SASP“利用系统提示辅助自动搜索”混为同一主机制。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="66" hidden="0" customHeight="1">
+      <x:c r="A24" s="142" t="str">
+        <x:v>数据提取</x:v>
+      </x:c>
+      <x:c r="B24" s="43" t="str">
+        <x:v>对抗媒体驱动的上下文/提示泄露</x:v>
+      </x:c>
+      <x:c r="C24" s="43" t="str">
+        <x:v>优化媒体去匹配“复述当前上下文”的行为函数，动态泄露系统提示或会话数据。</x:v>
+      </x:c>
+      <x:c r="D24" s="43" t="str">
+        <x:v>Image Hijacks—Leak Context</x:v>
+      </x:c>
+      <x:c r="E24" s="136" t="str">
+        <x:v>攻击目标是上下文/提示泄露，属于数据提取效果；与Image Hijacks的行为控制机制应分开，本版暂不纳入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="18" customHeight="1"/>
+    <x:row r="26" ht="18" customHeight="1"/>
+    <x:row r="27" ht="36" customHeight="1">
+      <x:c r="A27" s="121" t="str">
+        <x:v>新分类树：按模型实际利用的攻击机制组织</x:v>
+      </x:c>
+      <x:c r="B27" s="121"/>
+      <x:c r="C27" s="121"/>
+      <x:c r="D27" s="121"/>
+    </x:row>
+    <x:row r="28" ht="28" customHeight="1">
+      <x:c r="A28" s="125" t="str">
+        <x:v>二级分类统一按模型实际利用的攻击机制划分；本表作为方法库当前分类口径。</x:v>
+      </x:c>
+      <x:c r="B28" s="125"/>
+      <x:c r="C28" s="125"/>
+      <x:c r="D28" s="125"/>
+    </x:row>
+    <x:row r="29" ht="34" customHeight="1">
+      <x:c r="A29" s="131" t="str">
+        <x:v>一级分类</x:v>
+      </x:c>
+      <x:c r="B29" s="131" t="str">
+        <x:v>二级分类（攻击原理）</x:v>
+      </x:c>
+      <x:c r="C29" s="131" t="str">
+        <x:v>原理摘要</x:v>
+      </x:c>
+      <x:c r="D29" s="131" t="str">
+        <x:v>代表方法</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="82" customHeight="1">
+      <x:c r="A30" s="138" t="str">
+        <x:v>越狱</x:v>
+      </x:c>
+      <x:c r="B30" s="43" t="str">
         <x:v>视觉语义迁移与图像载荷</x:v>
       </x:c>
-      <x:c r="C5" s="86" t="str">
+      <x:c r="C30" s="43" t="str">
         <x:v>将完整危险语义或关键概念迁移到文字图、语义相关图或组合图中，利用视觉通道与文本通道安全对齐不一致。
 文本通常只保留通用执行引导。</x:v>
       </x:c>
-      <x:c r="D5" s="87" t="str">
+      <x:c r="D30" s="43" t="str">
         <x:v>FigStep、QR-Attack / Query-Relevant
 HADES（主归视觉载荷；含连续优化阶段）</x:v>
       </x:c>
-      <x:c r="E5" s="90" t="str">
-        <x:v>将原来的“视觉排版与跨模态语义载体”改为按实际机制命名：危险语义被迁移到图像或视觉文字中；保留 FigStep、QR-Attack 和 HADES。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="88" hidden="0" customHeight="1">
-      <x:c r="A6" s="92" t="str">
+    </x:row>
+    <x:row r="31" ht="82" customHeight="1">
+      <x:c r="A31" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B6" s="96" t="str">
+      <x:c r="B31" s="43" t="str">
         <x:v>跨模态/多图语义编码、拆分与重构</x:v>
       </x:c>
-      <x:c r="C6" s="96" t="str">
+      <x:c r="C31" s="43" t="str">
         <x:v>将危险线索编码或拆分到文本、图片、音频或多张图片中，使任一局部输入都不完整。
 模型需要解码、串联或重构后才能恢复完整意图。</x:v>
       </x:c>
-      <x:c r="D6" s="97" t="str">
+      <x:c r="D31" s="43" t="str">
         <x:v>MML、HIMRD、CrossTALK、DMN（主机制）
 Visual Object Replacement、SSJ、AdvBench-Omni
 MIR-SafetyBench—Complementarity</x:v>
       </x:c>
-      <x:c r="E6" s="100" t="str">
-        <x:v>扩展原“跨模态语义拆分与重组”，覆盖编码、拆分、引用和模型重构；纳入 MML、HIMRD、CrossTALK、DMN 主机制、Visual Object Replacement、SSJ、AdvBench-Omni 与 MIR-Complementarity。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="88" hidden="0" customHeight="1">
-      <x:c r="A7" s="92" t="str">
+    </x:row>
+    <x:row r="32" ht="82" customHeight="1">
+      <x:c r="A32" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B7" s="86" t="str">
+      <x:c r="B32" s="43" t="str">
         <x:v>输入结构变形与分布外绕过</x:v>
       </x:c>
-      <x:c r="C7" s="86" t="str">
+      <x:c r="C32" s="43" t="str">
         <x:v>在不改变核心攻击意图的情况下，通过打乱或变换内容表示，或者调整角色、特殊 Token、模态位置和轮次边界，使输入偏离模型安全对齐时的标准分布或模板结构。</x:v>
       </x:c>
-      <x:c r="D7" s="87" t="str">
+      <x:c r="D32" s="43" t="str">
         <x:v>SI-Attack、JOOD
 Role-Modality Attacks（RMA）</x:v>
       </x:c>
-      <x:c r="E7" s="90" t="str">
-        <x:v>从原混合类“视觉混淆、OOD与注意力分散”中拆出结构/OOD机制；SI-Attack、JOOD 以及仅改变角色、图像 Token 位置和模板边界的 RMA 归入此类。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="88" hidden="0" customHeight="1">
-      <x:c r="A8" s="92" t="str">
+    </x:row>
+    <x:row r="33" ht="82" customHeight="1">
+      <x:c r="A33" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B8" s="96" t="str">
+      <x:c r="B33" s="43" t="str">
         <x:v>注意力分散与任务干扰</x:v>
       </x:c>
-      <x:c r="C8" s="96" t="str">
+      <x:c r="C33" s="43" t="str">
         <x:v>使用对比内容、无害干扰项、递归引用、辅助子任务或数字链占用模型注意力，削弱其对完整危险意图的识别。</x:v>
       </x:c>
-      <x:c r="D8" s="97" t="str">
+      <x:c r="D33" s="43" t="str">
         <x:v>CS-DJ、Reference Attack
 MIR-SafetyBench—Relevance
 DMN—Number Chain（次要机制）</x:v>
       </x:c>
-      <x:c r="E8" s="100" t="str">
-        <x:v>把注意力占用与结构变形分开；CS-DJ、Reference Attack、MIR-Relevance 以及 DMN 的 Number Chain 次要机制归入此类。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="88" hidden="0" customHeight="1">
-      <x:c r="A9" s="92" t="str">
+    </x:row>
+    <x:row r="34" ht="82" customHeight="1">
+      <x:c r="A34" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B9" s="86" t="str">
+      <x:c r="B34" s="43" t="str">
         <x:v>角色扮演与情境/上下文诱导</x:v>
       </x:c>
-      <x:c r="C9" s="86" t="str">
+      <x:c r="C34" s="43" t="str">
         <x:v>利用角色身份、虚构故事、现实场景、权威语境或伪造对话历史，使危险请求在当前情境中显得合理。
 角色或上下文目标由此与安全目标竞争。</x:v>
       </x:c>
-      <x:c r="D9" s="87" t="str">
+      <x:c r="D34" s="43" t="str">
         <x:v>VRP、VoiceJailbreak、VisCo
 MIR-SafetyBench—Spatial Embedding</x:v>
       </x:c>
-      <x:c r="E9" s="90" t="str">
-        <x:v>从原“角色扮演、场景与推理链诱导”中拆出情境目标竞争机制；放 VRP、VoiceJailbreak、VisCo 与 MIR-Spatial Embedding。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="88" hidden="0" customHeight="1">
-      <x:c r="A10" s="92" t="str">
+    </x:row>
+    <x:row r="35" ht="82" customHeight="1">
+      <x:c r="A35" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B10" s="96" t="str">
+      <x:c r="B35" s="43" t="str">
         <x:v>结构化解题任务与推理链诱导</x:v>
       </x:c>
-      <x:c r="C10" s="96" t="str">
+      <x:c r="C35" s="43" t="str">
         <x:v>将危险任务包装成流程补全、分步求解、类比迁移、视觉恢复或目标驱动游戏。
 模型在执行既定解题流程时主动补出或重建危险内容。</x:v>
       </x:c>
-      <x:c r="D10" s="97" t="str">
+      <x:c r="D35" s="43" t="str">
         <x:v>FC-Attack、VisCRA、GAMBIT
 MIR-SafetyBench—Decomposition、Analogy</x:v>
       </x:c>
-      <x:c r="E10" s="100" t="str">
-        <x:v>把按既定流程解题、类比或推理链补全与角色情境分开；放 FC-Attack、VisCRA、GAMBIT，以及 MIR-Decomposition 和 Analogy。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="88" hidden="0" customHeight="1">
-      <x:c r="A11" s="92" t="str">
+    </x:row>
+    <x:row r="36" ht="82" customHeight="1">
+      <x:c r="A36" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B11" s="86" t="str">
+      <x:c r="B36" s="43" t="str">
         <x:v>时序推理</x:v>
       </x:c>
-      <x:c r="C11" s="86" t="str">
+      <x:c r="C36" s="43" t="str">
         <x:v>利用多张图片中的事件顺序和时间进展隐藏危险意图，要求模型理解连续过程或补全开始与结果之间的缺失步骤。</x:v>
       </x:c>
-      <x:c r="D11" s="87" t="str">
+      <x:c r="D36" s="43" t="str">
         <x:v>MIR-SafetyBench—Temporal Continuity
 MIR-SafetyBench—Temporal Jump</x:v>
       </x:c>
-      <x:c r="E11" s="90" t="str">
-        <x:v>MIR-SafetyBench 不再整体塞进一个大类；Temporal Continuity 与 Temporal Jump 单列，专门表示事件顺序理解和缺失步骤补全。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="88" hidden="0" customHeight="1">
-      <x:c r="A12" s="92" t="str">
+    </x:row>
+    <x:row r="37" ht="82" customHeight="1">
+      <x:c r="A37" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B12" s="96" t="str">
+      <x:c r="B37" s="43" t="str">
         <x:v>因果推理</x:v>
       </x:c>
-      <x:c r="C12" s="96" t="str">
+      <x:c r="C37" s="43" t="str">
         <x:v>展示危险结果并要求模型反推其形成原因或实现过程，使危险内容在因果推导完成后才显现。</x:v>
       </x:c>
-      <x:c r="D12" s="97" t="str">
+      <x:c r="D37" s="43" t="str">
         <x:v>MIR-SafetyBench—Causality</x:v>
       </x:c>
-      <x:c r="E12" s="100" t="str">
-        <x:v>将从结果反推形成过程的机制与普通时序补全分离；MIR-Causality 单列为因果推理。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="88" hidden="0" customHeight="1">
-      <x:c r="A13" s="92" t="str">
+    </x:row>
+    <x:row r="38" ht="82" customHeight="1">
+      <x:c r="A38" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B13" s="86" t="str">
+      <x:c r="B38" s="43" t="str">
         <x:v>空间场景关联推理</x:v>
       </x:c>
-      <x:c r="C13" s="86" t="str">
+      <x:c r="C38" s="43" t="str">
         <x:v>将相关线索分布在不同地点、视角或场景的图片中，要求模型推断这些场景之间未被直接展示的联系或行动。</x:v>
       </x:c>
-      <x:c r="D13" s="87" t="str">
+      <x:c r="D38" s="43" t="str">
         <x:v>MIR-SafetyBench—Spatial Juxtaposition</x:v>
       </x:c>
-      <x:c r="E13" s="90" t="str">
-        <x:v>将跨地点、视角或场景的关系推断与时间/因果推理分离；MIR-Spatial Juxtaposition 单列。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="88" hidden="0" customHeight="1">
-      <x:c r="A14" s="92" t="str">
+    </x:row>
+    <x:row r="39" ht="82" customHeight="1">
+      <x:c r="A39" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B14" s="96" t="str">
+      <x:c r="B39" s="43" t="str">
         <x:v>连续空间与多模态联合优化</x:v>
       </x:c>
-      <x:c r="C14" s="96" t="str">
+      <x:c r="C39" s="43" t="str">
         <x:v>在图像、音频、视觉嵌入等连续空间中优化对抗载荷，并可联合离散文本搜索或反馈改写，生成通用或定向越狱输入。</x:v>
       </x:c>
-      <x:c r="D14" s="97" t="str">
+      <x:c r="D39" s="43" t="str">
         <x:v>Visual-AE、Jailbreak in Pieces、imgJP
 UMK、BAP、GBJI、JAMA</x:v>
       </x:c>
-      <x:c r="E14" s="100" t="str">
-        <x:v>由“连续空间对抗优化”扩展为图像、音频和文本的联合优化；Visual-AE、Jailbreak in Pieces、imgJP、UMK、BAP、GBJI 与 JAMA 归入此类，JAMA 不再归入泛音频类。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="88" hidden="0" customHeight="1">
-      <x:c r="A15" s="92" t="str">
+    </x:row>
+    <x:row r="40" ht="82" customHeight="1">
+      <x:c r="A40" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B15" s="86" t="str">
+      <x:c r="B40" s="43" t="str">
         <x:v>训练投毒与后门触发</x:v>
       </x:c>
-      <x:c r="C15" s="86" t="str">
+      <x:c r="C40" s="43" t="str">
         <x:v>在视觉指令微调数据中注入恶意图文对，使模型学习图片与越狱行为的隐蔽关联，并在推理阶段由相同或相关图片触发。</x:v>
       </x:c>
-      <x:c r="D15" s="87" t="str">
+      <x:c r="D40" s="43" t="str">
         <x:v>ImgTrojan</x:v>
       </x:c>
-      <x:c r="E15" s="90" t="str">
-        <x:v>只保留真正发生在训练阶段的投毒/后门机制 ImgTrojan；依赖 Agent 记忆、检索和多智能体传播的 Agent Smith 移出模型级主表。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="88" hidden="0" customHeight="1">
-      <x:c r="A16" s="92" t="str">
+    </x:row>
+    <x:row r="41" ht="82" customHeight="1">
+      <x:c r="A41" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B16" s="96" t="str">
+      <x:c r="B41" s="43" t="str">
         <x:v>音频载荷与声学诱导</x:v>
       </x:c>
-      <x:c r="C16" s="96" t="str">
+      <x:c r="C41" s="43" t="str">
         <x:v>利用语言、口音、音色、韵律、语速、重音、噪声、无害音频干扰或近超声隐藏载荷，使人类感知、音频理解与模型安全判断之间出现不一致。</x:v>
       </x:c>
-      <x:c r="D16" s="97" t="str">
+      <x:c r="D41" s="43" t="str">
         <x:v>Multi-AudioJail、Jailbreak-AudioBench
 PJ-Break / AdvAudio-Prosody、AIA
 Sirens’ Whisper（SWhisper）</x:v>
       </x:c>
-      <x:c r="E16" s="100" t="str">
-        <x:v>集中表示语音载荷、韵律、口音、噪声、无害声学干扰和近超声载荷；放 Multi-AudioJail、Jailbreak-AudioBench、PJ-Break、AIA 与 SWhisper；VoiceJailbreak、JAMA 分别移到情境类和联合优化类。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="88" hidden="0" customHeight="1">
-      <x:c r="A17" s="92" t="str">
+    </x:row>
+    <x:row r="42" ht="82" customHeight="1">
+      <x:c r="A42" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B17" s="86" t="str">
+      <x:c r="B42" s="43" t="str">
         <x:v>模态迁移与冗余语义承载</x:v>
       </x:c>
-      <x:c r="C17" s="86" t="str">
+      <x:c r="C42" s="43" t="str">
         <x:v>把既有文本攻击或同一危险语义转换到图片、音频及其组合中，或在多个模态中重复承载同一关键词，利用不同模态间的安全不一致。</x:v>
       </x:c>
-      <x:c r="D17" s="87" t="str">
+      <x:c r="D42" s="43" t="str">
         <x:v>The Alignment Curse
 Omni-SafetyBench（纯音频、图+文、文+音、文+图+音子集）</x:v>
       </x:c>
-      <x:c r="E17" s="90" t="str">
-        <x:v>新增分类以区分两种机制：既有文本攻击直接迁移到音频，以及同一危险短语在图片、音频中冗余承载；对应 The Alignment Curse 与 Omni-SafetyBench。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="88" hidden="0" customHeight="1">
-      <x:c r="A18" s="92" t="str">
+    </x:row>
+    <x:row r="43" ht="82" customHeight="1">
+      <x:c r="A43" s="138" t="str">
         <x:v>越狱</x:v>
       </x:c>
-      <x:c r="B18" s="96" t="str">
+      <x:c r="B43" s="43" t="str">
         <x:v>自动化提示优化与反馈搜索</x:v>
       </x:c>
-      <x:c r="C18" s="96" t="str">
+      <x:c r="C43" s="43" t="str">
         <x:v>使用红队模型自动生成候选越狱提示，并依据目标模型的回答、成功评分或失败反馈持续筛选和改写。
 部分方法还利用已知或推断的系统提示与防御规则，提高优化的针对性。</x:v>
       </x:c>
-      <x:c r="D18" s="97" t="str">
+      <x:c r="D43" s="43" t="str">
         <x:v>SASP、AutoJailbreak</x:v>
       </x:c>
-      <x:c r="E18" s="100" t="str">
-        <x:v>SASP 与 AutoJailbreak 的核心都是自动生成候选、评估回答并迭代改写，因此合并；SASP 的系统提示利用仅作为辅助信息标签。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="88" hidden="0" customHeight="1">
-      <x:c r="A19" s="102" t="str">
+    </x:row>
+    <x:row r="44" ht="82" customHeight="1">
+      <x:c r="A44" s="140" t="str">
         <x:v>提示注入</x:v>
       </x:c>
-      <x:c r="B19" s="86" t="str">
+      <x:c r="B44" s="43" t="str">
         <x:v>显式视觉/音频载荷</x:v>
       </x:c>
-      <x:c r="C19" s="86" t="str">
+      <x:c r="C44" s="43" t="str">
         <x:v>把人类、OCR或ASR能够直接识别的自然语言命令写入图片或声音中，使模型把媒体内容误当成应执行的指令。</x:v>
       </x:c>
-      <x:c r="D19" s="87" t="str">
+      <x:c r="D44" s="43" t="str">
         <x:v>Visual OCR Injection〔攻击模式〕
 Audible Instruction〔攻击模式〕</x:v>
       </x:c>
-      <x:c r="E19" s="90" t="str">
-        <x:v>保留并明确 OCR/ASR 内容被错误当成可执行指令这一机制；当前范围仅研究图、文、音频，因此移除 Video-frame Instruction。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="88" hidden="0" customHeight="1">
-      <x:c r="A20" s="102" t="str">
+    </x:row>
+    <x:row r="45" ht="82" customHeight="1">
+      <x:c r="A45" s="140" t="str">
         <x:v>提示注入</x:v>
       </x:c>
-      <x:c r="B20" s="96" t="str">
+      <x:c r="B45" s="43" t="str">
         <x:v>隐蔽呈现与感知/预处理差异</x:v>
       </x:c>
-      <x:c r="C20" s="96" t="str">
+      <x:c r="C45" s="43" t="str">
         <x:v>指令仍以文字形式存在，但通过低对比度、背景适配、透视变形或缩放后显现等方式降低人类与传统检测器的可见性，同时保留模型可读性。</x:v>
       </x:c>
-      <x:c r="D20" s="97" t="str">
+      <x:c r="D45" s="43" t="str">
         <x:v>Image-based Prompt Injection（IPI）
 InkJect、Anamorpher / Image Scaling Attack</x:v>
       </x:c>
-      <x:c r="E20" s="100" t="str">
-        <x:v>从原“隐式对抗扰动与语义碰撞”拆出感知差异类：InkJect、Anamorpher、IPI 的完整文字仍存在，只是借低对比度、透视或缩放制造人、检测器与模型之间的可见性差异。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="88" hidden="0" customHeight="1">
-      <x:c r="A21" s="102" t="str">
+    </x:row>
+    <x:row r="46" ht="82" customHeight="1">
+      <x:c r="A46" s="140" t="str">
         <x:v>提示注入</x:v>
       </x:c>
-      <x:c r="B21" s="86" t="str">
+      <x:c r="B46" s="43" t="str">
         <x:v>视觉语义编码</x:v>
       </x:c>
-      <x:c r="C21" s="86" t="str">
+      <x:c r="C46" s="43" t="str">
         <x:v>不直接写出完整自然语言命令，而是利用图标组合、Rebus图谜和视觉双关，让模型通过视觉推理恢复隐藏指令。</x:v>
       </x:c>
-      <x:c r="D21" s="87" t="str">
+      <x:c r="D46" s="43" t="str">
         <x:v>NVIDIA Semantic / Rebus Visual Prompt Injection</x:v>
       </x:c>
-      <x:c r="E21" s="90" t="str">
-        <x:v>NVIDIA Rebus 不隐藏完整文字也不做梯度扰动，而是让模型从图标、图谜和视觉双关中恢复指令，因此单列。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="88" hidden="0" customHeight="1">
-      <x:c r="A22" s="102" t="str">
+    </x:row>
+    <x:row r="47" ht="82" customHeight="1">
+      <x:c r="A47" s="140" t="str">
         <x:v>提示注入</x:v>
       </x:c>
-      <x:c r="B22" s="96" t="str">
+      <x:c r="B47" s="43" t="str">
         <x:v>对抗扰动与表示/行为对齐</x:v>
       </x:c>
-      <x:c r="C22" s="96" t="str">
+      <x:c r="C47" s="43" t="str">
         <x:v>优化图像或音频连续空间，使输入匹配攻击者指定的输出行为、提示语义、跨模态特征或融合层隐藏状态。
 多轮持续污染作为攻击效果标签，不另设二级分类。</x:v>
       </x:c>
-      <x:c r="D22" s="97" t="str">
+      <x:c r="D47" s="43" t="str">
         <x:v>Adversarial Instruction Blending（含 Dialog Poisoning）
 Image Hijacks—Prompt/Behaviour Matching
 Covert Visual Prompt Injection（原 AdvPIA）、CrossMPI</x:v>
       </x:c>
-      <x:c r="E22" s="100" t="str">
-        <x:v>Instruction Blending、Image Hijacks、AdvPIA、CrossMPI 都通过连续空间优化对齐到目标提示语义、隐藏表示、融合状态或输出行为；Dialog Poisoning 的持续污染仅作为多轮效果/持久性标签。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
-      <x:c r="A23" s="16"/>
-      <x:c r="B23" s="16"/>
-      <x:c r="C23" s="16"/>
-      <x:c r="D23" s="17"/>
-    </x:row>
-    <x:row r="24" ht="52" hidden="0" customHeight="1">
-      <x:c r="A24" s="116" t="str">
-        <x:v>范围调整：元数据/外部资源间接注入、跨模态代理与工具劫持主要描述网页、邮件、附件、知识库、Agent 决策和工具调用等应用链路，本版移出主表；数据提取方向暂不纳入。最终主表仅保留越狱与提示注入。</x:v>
-      </x:c>
-      <x:c r="B24" s="116"/>
-      <x:c r="C24" s="116"/>
-      <x:c r="D24" s="117"/>
-      <x:c r="E24" s="115"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
     <x:mergeCell ref="A2:E2"/>
-    <x:mergeCell ref="A24:E24"/>
+    <x:mergeCell ref="A27:D27"/>
+    <x:mergeCell ref="A28:D28"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A5:A24">
     <x:cfRule type="containsText" dxfId="9" priority="2" aboveAverage="0" percent="0" bottom="0" operator="containsText" text="越狱" rank="0" equalAverage="0">
@@ -4943,8 +5412,9 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4aadd356db464bf4"/>
+  <x:tableParts count="2">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4ce4eeb67594ddc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R773e56646ef24015"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4993,28 +5463,28 @@
   <x:sheetData>
     <x:row r="1" ht="36" hidden="0" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E1" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F1" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G1" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H1" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="I1" s="18"/>
       <x:c r="J1" s="18"/>
@@ -5052,25 +5522,25 @@
         <x:v>共52条：越狱41条、提示注入11条；仅保留图、文、音频范围，机制与来源复核截至2026-08-26。</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="G2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="H2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" hidden="0" customHeight="1">
@@ -11497,7 +11967,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0538fb33a8d4915"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6f0422081194973"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11518,1264 +11988,1264 @@
   <x:sheetData>
     <x:row r="1" ht="36" hidden="0" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E1" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F1" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G1" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="H1" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="I1" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" hidden="0" customHeight="1">
       <x:c r="A2" s="27" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B2" s="27" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C2" s="27" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D2" s="27" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E2" s="27" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F2" s="27" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="G2" s="27" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="H2" s="27" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="14.25" hidden="0">
       <x:c r="A4" s="28" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B4" s="28" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="B4" s="28" t="s">
+      <x:c r="C4" s="28" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C4" s="28" t="s">
+      <x:c r="D4" s="28" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="D4" s="28" t="s">
+      <x:c r="E4" s="28" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="E4" s="28" t="s">
+      <x:c r="F4" s="28" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="F4" s="28" t="s">
+      <x:c r="G4" s="28" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="G4" s="28" t="s">
+      <x:c r="H4" s="28" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="H4" s="28" t="s">
+      <x:c r="I4" s="28" t="s">
         <x:v>33</x:v>
-      </x:c>
-      <x:c r="I4" s="28" t="s">
-        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="70" hidden="0" customHeight="1">
       <x:c r="A5" s="29" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B5" s="29" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="B5" s="29" t="s">
+      <x:c r="C5" s="29" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="C5" s="29" t="s">
+      <x:c r="D5" s="29" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="D5" s="29" t="s">
+      <x:c r="E5" s="29" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="E5" s="29" t="s">
+      <x:c r="F5" s="30" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="F5" s="30" t="s">
+      <x:c r="G5" s="29" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="G5" s="29" t="s">
+      <x:c r="H5" s="30" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="H5" s="30" t="s">
+      <x:c r="I5" s="30" t="s">
         <x:v>42</x:v>
-      </x:c>
-      <x:c r="I5" s="30" t="s">
-        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="70" hidden="0" customHeight="1">
       <x:c r="A6" s="29" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B6" s="29" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="B6" s="29" t="s">
+      <x:c r="C6" s="29" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D6" s="29" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="C6" s="29" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="D6" s="29" t="s">
+      <x:c r="E6" s="29" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="E6" s="29" t="s">
+      <x:c r="F6" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G6" s="29" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="F6" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G6" s="29" t="s">
+      <x:c r="H6" s="30" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="H6" s="30" t="s">
+      <x:c r="I6" s="30" t="s">
         <x:v>49</x:v>
-      </x:c>
-      <x:c r="I6" s="30" t="s">
-        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="70" hidden="0" customHeight="1">
       <x:c r="A7" s="29" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B7" s="29" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="B7" s="29" t="s">
+      <x:c r="C7" s="29" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D7" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E7" s="29" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="C7" s="29" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="D7" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E7" s="29" t="s">
+      <x:c r="F7" s="30" t="s">
         <x:v>53</x:v>
-      </x:c>
-      <x:c r="F7" s="30" t="s">
-        <x:v>54</x:v>
       </x:c>
       <x:c r="G7" s="30"/>
       <x:c r="H7" s="30" t="s">
-        <x:v>49</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="I7" s="30" t="s">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="70" hidden="0" customHeight="1">
       <x:c r="A8" s="29" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="B8" s="29" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="B8" s="29" t="s">
+      <x:c r="C8" s="29" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D8" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E8" s="29" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="C8" s="29" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="D8" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E8" s="29" t="s">
+      <x:c r="F8" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G8" s="29" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="F8" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G8" s="29" t="s">
+      <x:c r="H8" s="30" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="H8" s="30" t="s">
+      <x:c r="I8" s="30" t="s">
         <x:v>60</x:v>
-      </x:c>
-      <x:c r="I8" s="30" t="s">
-        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="70" hidden="0" customHeight="1">
       <x:c r="A9" s="29" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B9" s="29" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="B9" s="29" t="s">
+      <x:c r="C9" s="29" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D9" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E9" s="29" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="C9" s="29" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="D9" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E9" s="29" t="s">
+      <x:c r="F9" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G9" s="29" t="s">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="F9" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G9" s="29" t="s">
+      <x:c r="H9" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I9" s="30" t="s">
         <x:v>65</x:v>
-      </x:c>
-      <x:c r="H9" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I9" s="30" t="s">
-        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="70" hidden="0" customHeight="1">
       <x:c r="A10" s="29" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="B10" s="29" t="s">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="B10" s="29" t="s">
+      <x:c r="C10" s="29" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D10" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E10" s="29" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="C10" s="29" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="D10" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E10" s="29" t="s">
+      <x:c r="F10" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G10" s="29" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="F10" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G10" s="29" t="s">
+      <x:c r="H10" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I10" s="30" t="s">
         <x:v>70</x:v>
-      </x:c>
-      <x:c r="H10" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I10" s="30" t="s">
-        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="70" hidden="0" customHeight="1">
       <x:c r="A11" s="29" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B11" s="29" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C11" s="29" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D11" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E11" s="29" t="s">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="B11" s="29" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="C11" s="29" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="D11" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E11" s="29" t="s">
-        <x:v>73</x:v>
-      </x:c>
       <x:c r="F11" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G11" s="30"/>
       <x:c r="H11" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I11" s="30" t="s">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="70" hidden="0" customHeight="1">
       <x:c r="A12" s="29" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="B12" s="29" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="B12" s="29" t="s">
+      <x:c r="C12" s="29" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D12" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E12" s="29" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="C12" s="29" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="D12" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E12" s="29" t="s">
+      <x:c r="F12" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G12" s="29" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="F12" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G12" s="29" t="s">
+      <x:c r="H12" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I12" s="29" t="s">
         <x:v>78</x:v>
-      </x:c>
-      <x:c r="H12" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I12" s="29" t="s">
-        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="70" hidden="0" customHeight="1">
       <x:c r="A13" s="29" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="B13" s="29" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="B13" s="29" t="s">
+      <x:c r="C13" s="29" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D13" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E13" s="29" t="s">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="C13" s="29" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="D13" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E13" s="29" t="s">
+      <x:c r="F13" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G13" s="29" t="s">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="F13" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G13" s="29" t="s">
+      <x:c r="H13" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I13" s="30" t="s">
         <x:v>83</x:v>
-      </x:c>
-      <x:c r="H13" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I13" s="30" t="s">
-        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="70" hidden="0" customHeight="1">
       <x:c r="A14" s="29" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="B14" s="29" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="C14" s="29" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="B14" s="29" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="C14" s="29" t="s">
+      <x:c r="D14" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E14" s="29" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="D14" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E14" s="29" t="s">
+      <x:c r="F14" s="30" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="F14" s="30" t="s">
+      <x:c r="G14" s="29" t="s">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="G14" s="29" t="s">
+      <x:c r="H14" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I14" s="30" t="s">
         <x:v>89</x:v>
-      </x:c>
-      <x:c r="H14" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I14" s="30" t="s">
-        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="70" hidden="0" customHeight="1">
       <x:c r="A15" s="29" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="B15" s="29" t="s">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="B15" s="29" t="s">
+      <x:c r="C15" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D15" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E15" s="29" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="C15" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D15" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E15" s="29" t="s">
-        <x:v>93</x:v>
-      </x:c>
       <x:c r="F15" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G15" s="30"/>
       <x:c r="H15" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I15" s="30" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="70" hidden="0" customHeight="1">
       <x:c r="A16" s="29" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="B16" s="29" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C16" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D16" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E16" s="29" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="B16" s="29" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="C16" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D16" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E16" s="29" t="s">
+      <x:c r="F16" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G16" s="29" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="F16" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G16" s="29" t="s">
+      <x:c r="H16" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I16" s="30" t="s">
         <x:v>97</x:v>
-      </x:c>
-      <x:c r="H16" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I16" s="30" t="s">
-        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="70" hidden="0" customHeight="1">
       <x:c r="A17" s="29" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B17" s="29" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C17" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D17" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E17" s="29" t="s">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="B17" s="29" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="C17" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D17" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E17" s="29" t="s">
+      <x:c r="F17" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G17" s="29" t="s">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="F17" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G17" s="29" t="s">
+      <x:c r="H17" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I17" s="30" t="s">
         <x:v>101</x:v>
-      </x:c>
-      <x:c r="H17" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I17" s="30" t="s">
-        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="70" hidden="0" customHeight="1">
       <x:c r="A18" s="29" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B18" s="29" t="s">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="B18" s="29" t="s">
+      <x:c r="C18" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D18" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E18" s="29" t="s">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="C18" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D18" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E18" s="29" t="s">
+      <x:c r="F18" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G18" s="29" t="s">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="F18" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G18" s="29" t="s">
+      <x:c r="H18" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I18" s="30" t="s">
         <x:v>106</x:v>
-      </x:c>
-      <x:c r="H18" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I18" s="30" t="s">
-        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="70" hidden="0" customHeight="1">
       <x:c r="A19" s="29" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="B19" s="29" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C19" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D19" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E19" s="29" t="s">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="B19" s="29" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="C19" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D19" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E19" s="29" t="s">
-        <x:v>109</x:v>
-      </x:c>
       <x:c r="F19" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G19" s="30"/>
       <x:c r="H19" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I19" s="30" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="70" hidden="0" customHeight="1">
       <x:c r="A20" s="29" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="B20" s="29" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C20" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D20" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E20" s="29" t="s">
         <x:v>111</x:v>
       </x:c>
-      <x:c r="B20" s="29" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="C20" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D20" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E20" s="29" t="s">
+      <x:c r="F20" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G20" s="29" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="F20" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G20" s="29" t="s">
+      <x:c r="H20" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I20" s="30" t="s">
         <x:v>113</x:v>
-      </x:c>
-      <x:c r="H20" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I20" s="30" t="s">
-        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="70" hidden="0" customHeight="1">
       <x:c r="A21" s="29" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="B21" s="29" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C21" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D21" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E21" s="29" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="B21" s="29" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="C21" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D21" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E21" s="29" t="s">
+      <x:c r="F21" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G21" s="29" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="F21" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G21" s="29" t="s">
+      <x:c r="H21" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I21" s="30" t="s">
         <x:v>117</x:v>
-      </x:c>
-      <x:c r="H21" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I21" s="30" t="s">
-        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="70" hidden="0" customHeight="1">
       <x:c r="A22" s="29" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="B22" s="29" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C22" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D22" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E22" s="29" t="s">
         <x:v>119</x:v>
       </x:c>
-      <x:c r="B22" s="29" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="C22" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D22" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E22" s="29" t="s">
+      <x:c r="F22" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G22" s="29" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="F22" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G22" s="29" t="s">
+      <x:c r="H22" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I22" s="30" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="H22" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I22" s="30" t="s">
-        <x:v>122</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="70" hidden="0" customHeight="1">
       <x:c r="A23" s="29" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="B23" s="29" t="s">
         <x:v>123</x:v>
       </x:c>
-      <x:c r="B23" s="29" t="s">
+      <x:c r="C23" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D23" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E23" s="29" t="s">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="C23" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D23" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E23" s="29" t="s">
+      <x:c r="F23" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G23" s="29" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="F23" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G23" s="29" t="s">
+      <x:c r="H23" s="30" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="I23" s="30" t="s">
         <x:v>126</x:v>
-      </x:c>
-      <x:c r="H23" s="30" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="I23" s="30" t="s">
-        <x:v>127</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="70" hidden="0" customHeight="1">
       <x:c r="A24" s="29" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="B24" s="29" t="s">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="B24" s="29" t="s">
+      <x:c r="C24" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D24" s="29" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="C24" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D24" s="29" t="s">
+      <x:c r="E24" s="29" t="s">
         <x:v>130</x:v>
       </x:c>
-      <x:c r="E24" s="29" t="s">
+      <x:c r="F24" s="30" t="s">
         <x:v>131</x:v>
-      </x:c>
-      <x:c r="F24" s="30" t="s">
-        <x:v>132</x:v>
       </x:c>
       <x:c r="G24" s="30"/>
       <x:c r="H24" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I24" s="30" t="s">
-        <x:v>133</x:v>
+        <x:v>132</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="70" hidden="0" customHeight="1">
       <x:c r="A25" s="29" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="B25" s="29" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C25" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D25" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E25" s="29" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="B25" s="29" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="C25" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D25" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E25" s="29" t="s">
-        <x:v>135</x:v>
-      </x:c>
       <x:c r="F25" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G25" s="30"/>
       <x:c r="H25" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I25" s="30" t="s">
-        <x:v>136</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="70" hidden="0" customHeight="1">
       <x:c r="A26" s="29" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="B26" s="29" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C26" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D26" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E26" s="29" t="s">
         <x:v>137</x:v>
       </x:c>
-      <x:c r="B26" s="29" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="C26" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D26" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E26" s="29" t="s">
+      <x:c r="F26" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G26" s="29" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="F26" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G26" s="29" t="s">
+      <x:c r="H26" s="30" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="H26" s="30" t="s">
+      <x:c r="I26" s="30" t="s">
         <x:v>140</x:v>
-      </x:c>
-      <x:c r="I26" s="30" t="s">
-        <x:v>141</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="70" hidden="0" customHeight="1">
       <x:c r="A27" s="29" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="B27" s="29" t="s">
         <x:v>142</x:v>
       </x:c>
-      <x:c r="B27" s="29" t="s">
+      <x:c r="C27" s="29" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D27" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E27" s="29" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="C27" s="29" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D27" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E27" s="29" t="s">
+      <x:c r="F27" s="30" t="s">
         <x:v>144</x:v>
       </x:c>
-      <x:c r="F27" s="30" t="s">
+      <x:c r="G27" s="29" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="G27" s="29" t="s">
+      <x:c r="H27" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I27" s="30" t="s">
         <x:v>146</x:v>
-      </x:c>
-      <x:c r="H27" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I27" s="30" t="s">
-        <x:v>147</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="70" hidden="0" customHeight="1">
       <x:c r="A28" s="29" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="B28" s="29" t="s">
         <x:v>148</x:v>
       </x:c>
-      <x:c r="B28" s="29" t="s">
+      <x:c r="C28" s="29" t="s">
         <x:v>149</x:v>
       </x:c>
-      <x:c r="C28" s="29" t="s">
+      <x:c r="D28" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E28" s="29" t="s">
         <x:v>150</x:v>
       </x:c>
-      <x:c r="D28" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E28" s="29" t="s">
+      <x:c r="F28" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G28" s="29" t="s">
         <x:v>151</x:v>
       </x:c>
-      <x:c r="F28" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G28" s="29" t="s">
+      <x:c r="H28" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I28" s="30" t="s">
         <x:v>152</x:v>
-      </x:c>
-      <x:c r="H28" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I28" s="30" t="s">
-        <x:v>153</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="70" hidden="0" customHeight="1">
       <x:c r="A29" s="29" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="B29" s="29" t="s">
         <x:v>154</x:v>
       </x:c>
-      <x:c r="B29" s="29" t="s">
+      <x:c r="C29" s="29" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="D29" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E29" s="29" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="C29" s="29" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="D29" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E29" s="29" t="s">
-        <x:v>156</x:v>
-      </x:c>
       <x:c r="F29" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G29" s="30"/>
       <x:c r="H29" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I29" s="30" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="70" hidden="0" customHeight="1">
       <x:c r="A30" s="29" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="B30" s="29" t="s">
         <x:v>158</x:v>
       </x:c>
-      <x:c r="B30" s="29" t="s">
+      <x:c r="C30" s="29" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="D30" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E30" s="29" t="s">
         <x:v>159</x:v>
       </x:c>
-      <x:c r="C30" s="29" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="D30" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E30" s="29" t="s">
+      <x:c r="F30" s="30" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="G30" s="29" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="H30" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I30" s="30" t="s">
         <x:v>160</x:v>
-      </x:c>
-      <x:c r="F30" s="30" t="s">
-        <x:v>145</x:v>
-      </x:c>
-      <x:c r="G30" s="29" t="s">
-        <x:v>146</x:v>
-      </x:c>
-      <x:c r="H30" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I30" s="30" t="s">
-        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="70" hidden="0" customHeight="1">
       <x:c r="A31" s="29" t="s">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="B31" s="29" t="s">
         <x:v>162</x:v>
       </x:c>
-      <x:c r="B31" s="29" t="s">
+      <x:c r="C31" s="29" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="D31" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E31" s="29" t="s">
         <x:v>163</x:v>
       </x:c>
-      <x:c r="C31" s="29" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="D31" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E31" s="29" t="s">
-        <x:v>164</x:v>
-      </x:c>
       <x:c r="F31" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G31" s="30"/>
       <x:c r="H31" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I31" s="30" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="70" hidden="0" customHeight="1">
       <x:c r="A32" s="29" t="s">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="B32" s="29" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="C32" s="29" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="D32" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E32" s="29" t="s">
         <x:v>166</x:v>
       </x:c>
-      <x:c r="B32" s="29" t="s">
-        <x:v>163</x:v>
-      </x:c>
-      <x:c r="C32" s="29" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="D32" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E32" s="29" t="s">
+      <x:c r="F32" s="30" t="s">
         <x:v>167</x:v>
-      </x:c>
-      <x:c r="F32" s="30" t="s">
-        <x:v>168</x:v>
       </x:c>
       <x:c r="G32" s="30"/>
       <x:c r="H32" s="30" t="s">
-        <x:v>140</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="I32" s="30" t="s">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="70" hidden="0" customHeight="1">
       <x:c r="A33" s="29" t="s">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="B33" s="30" t="s">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="B33" s="30" t="s">
+      <x:c r="C33" s="29" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="D33" s="29" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="E33" s="29" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="C33" s="29" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="D33" s="29" t="s">
-        <x:v>130</x:v>
-      </x:c>
-      <x:c r="E33" s="29" t="s">
-        <x:v>172</x:v>
-      </x:c>
       <x:c r="F33" s="30" t="s">
-        <x:v>132</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="G33" s="30"/>
       <x:c r="H33" s="30" t="s">
-        <x:v>140</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="I33" s="30" t="s">
-        <x:v>173</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="70" hidden="0" customHeight="1">
       <x:c r="A34" s="29" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="B34" s="29" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="C34" s="29" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="D34" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E34" s="29" t="s">
         <x:v>174</x:v>
       </x:c>
-      <x:c r="B34" s="29" t="s">
-        <x:v>163</x:v>
-      </x:c>
-      <x:c r="C34" s="29" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="D34" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E34" s="29" t="s">
+      <x:c r="F34" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G34" s="29" t="s">
         <x:v>175</x:v>
       </x:c>
-      <x:c r="F34" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G34" s="29" t="s">
+      <x:c r="H34" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I34" s="30" t="s">
         <x:v>176</x:v>
-      </x:c>
-      <x:c r="H34" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I34" s="30" t="s">
-        <x:v>177</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="70" hidden="0" customHeight="1">
       <x:c r="A35" s="29" t="s">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="B35" s="29" t="s">
         <x:v>178</x:v>
       </x:c>
-      <x:c r="B35" s="29" t="s">
+      <x:c r="C35" s="29" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="D35" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E35" s="29" t="s">
         <x:v>179</x:v>
       </x:c>
-      <x:c r="C35" s="29" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="D35" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E35" s="29" t="s">
-        <x:v>180</x:v>
-      </x:c>
       <x:c r="F35" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G35" s="30"/>
       <x:c r="H35" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I35" s="30" t="s">
-        <x:v>181</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="70" hidden="0" customHeight="1">
       <x:c r="A36" s="29" t="s">
+        <x:v>181</x:v>
+      </x:c>
+      <x:c r="B36" s="29" t="s">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="C36" s="29" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="D36" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E36" s="29" t="s">
         <x:v>182</x:v>
       </x:c>
-      <x:c r="B36" s="29" t="s">
-        <x:v>179</x:v>
-      </x:c>
-      <x:c r="C36" s="29" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="D36" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E36" s="29" t="s">
-        <x:v>183</x:v>
-      </x:c>
       <x:c r="F36" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G36" s="30"/>
       <x:c r="H36" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I36" s="30" t="s">
-        <x:v>184</x:v>
+        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="70" hidden="0" customHeight="1">
       <x:c r="A37" s="29" t="s">
+        <x:v>184</x:v>
+      </x:c>
+      <x:c r="B37" s="29" t="s">
         <x:v>185</x:v>
       </x:c>
-      <x:c r="B37" s="29" t="s">
+      <x:c r="C37" s="29" t="s">
         <x:v>186</x:v>
       </x:c>
-      <x:c r="C37" s="29" t="s">
+      <x:c r="D37" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E37" s="29" t="s">
         <x:v>187</x:v>
       </x:c>
-      <x:c r="D37" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E37" s="29" t="s">
-        <x:v>188</x:v>
-      </x:c>
       <x:c r="F37" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G37" s="30"/>
       <x:c r="H37" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I37" s="30" t="s">
-        <x:v>189</x:v>
+        <x:v>188</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="70" hidden="0" customHeight="1">
       <x:c r="A38" s="29" t="s">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="B38" s="29" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="C38" s="29" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="D38" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E38" s="29" t="s">
         <x:v>190</x:v>
       </x:c>
-      <x:c r="B38" s="29" t="s">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="C38" s="29" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="D38" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E38" s="29" t="s">
-        <x:v>191</x:v>
-      </x:c>
       <x:c r="F38" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G38" s="30"/>
       <x:c r="H38" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I38" s="30" t="s">
-        <x:v>192</x:v>
+        <x:v>191</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="70" hidden="0" customHeight="1">
       <x:c r="A39" s="29" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="B39" s="29" t="s">
         <x:v>193</x:v>
       </x:c>
-      <x:c r="B39" s="29" t="s">
+      <x:c r="C39" s="29" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="D39" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E39" s="29" t="s">
         <x:v>194</x:v>
       </x:c>
-      <x:c r="C39" s="29" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="D39" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E39" s="29" t="s">
+      <x:c r="F39" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G39" s="29" t="s">
         <x:v>195</x:v>
       </x:c>
-      <x:c r="F39" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G39" s="29" t="s">
+      <x:c r="H39" s="30" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I39" s="30" t="s">
         <x:v>196</x:v>
-      </x:c>
-      <x:c r="H39" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I39" s="30" t="s">
-        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="70" hidden="0" customHeight="1">
       <x:c r="A40" s="29" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="B40" s="29" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="C40" s="29" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="D40" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E40" s="29" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="B40" s="29" t="s">
-        <x:v>194</x:v>
-      </x:c>
-      <x:c r="C40" s="29" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="D40" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E40" s="29" t="s">
-        <x:v>199</x:v>
-      </x:c>
       <x:c r="F40" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G40" s="30"/>
       <x:c r="H40" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I40" s="30" t="s">
-        <x:v>200</x:v>
+        <x:v>199</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="70" hidden="0" customHeight="1">
       <x:c r="A41" s="29" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="B41" s="29" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="C41" s="29" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="D41" s="29" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E41" s="29" t="s">
         <x:v>201</x:v>
       </x:c>
-      <x:c r="B41" s="29" t="s">
-        <x:v>194</x:v>
-      </x:c>
-      <x:c r="C41" s="29" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="D41" s="29" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="E41" s="29" t="s">
-        <x:v>202</x:v>
-      </x:c>
       <x:c r="F41" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G41" s="30"/>
       <x:c r="H41" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I41" s="30" t="s">
-        <x:v>203</x:v>
+        <x:v>202</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="70" hidden="0" customHeight="1">
       <x:c r="A42" s="29" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="B42" s="29" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="C42" s="29" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="D42" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E42" s="29" t="s">
         <x:v>204</x:v>
       </x:c>
-      <x:c r="B42" s="29" t="s">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="C42" s="29" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="D42" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E42" s="29" t="s">
-        <x:v>205</x:v>
-      </x:c>
       <x:c r="F42" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G42" s="30"/>
       <x:c r="H42" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I42" s="30" t="s">
-        <x:v>206</x:v>
+        <x:v>205</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="70" hidden="0" customHeight="1">
       <x:c r="A43" s="29" t="s">
+        <x:v>206</x:v>
+      </x:c>
+      <x:c r="B43" s="29" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="C43" s="29" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="D43" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E43" s="29" t="s">
         <x:v>207</x:v>
       </x:c>
-      <x:c r="B43" s="29" t="s">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="C43" s="29" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="D43" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E43" s="29" t="s">
-        <x:v>208</x:v>
-      </x:c>
       <x:c r="F43" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G43" s="30"/>
       <x:c r="H43" s="30" t="s">
-        <x:v>42</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="I43" s="30" t="s">
-        <x:v>209</x:v>
+        <x:v>208</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="70" hidden="0" customHeight="1">
       <x:c r="A44" s="29" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="B44" s="29" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="C44" s="29" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="D44" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E44" s="29" t="s">
         <x:v>210</x:v>
       </x:c>
-      <x:c r="B44" s="29" t="s">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="C44" s="29" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="D44" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E44" s="29" t="s">
+      <x:c r="F44" s="30" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G44" s="29" t="s">
         <x:v>211</x:v>
       </x:c>
-      <x:c r="F44" s="30" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G44" s="29" t="s">
+      <x:c r="H44" s="30" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="I44" s="30" t="s">
         <x:v>212</x:v>
-      </x:c>
-      <x:c r="H44" s="30" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="I44" s="30" t="s">
-        <x:v>213</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="70" hidden="0" customHeight="1">
       <x:c r="A45" s="29" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="B45" s="29" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="C45" s="29" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="D45" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E45" s="29" t="s">
         <x:v>214</x:v>
       </x:c>
-      <x:c r="B45" s="29" t="s">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="C45" s="29" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="D45" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E45" s="29" t="s">
-        <x:v>215</x:v>
-      </x:c>
       <x:c r="F45" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G45" s="30"/>
       <x:c r="H45" s="30" t="s">
-        <x:v>140</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="I45" s="30" t="s">
-        <x:v>216</x:v>
+        <x:v>215</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="70" hidden="0" customHeight="1">
       <x:c r="A46" s="29" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="B46" s="29" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="C46" s="29" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="D46" s="29" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E46" s="29" t="s">
         <x:v>217</x:v>
       </x:c>
-      <x:c r="B46" s="29" t="s">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="C46" s="29" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="D46" s="29" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E46" s="29" t="s">
-        <x:v>218</x:v>
-      </x:c>
       <x:c r="F46" s="30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G46" s="30"/>
       <x:c r="H46" s="30" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I46" s="30" t="s">
-        <x:v>219</x:v>
+        <x:v>218</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12796,7 +13266,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6873544494f4993"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e5b4ec526a0444a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12811,49 +13281,49 @@
   <x:sheetData>
     <x:row r="1" ht="36" hidden="0" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>220</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>220</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>221</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>221</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
-        <x:v>221</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="D2" s="2" t="s">
-        <x:v>221</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
-        <x:v>221</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="F2" s="2" t="s">
-        <x:v>221</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="G2" s="2" t="s">
-        <x:v>221</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="H2" s="2" t="s">
-        <x:v>221</x:v>
+        <x:v>220</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="14.25" hidden="0">
       <x:c r="A4" s="31" t="s">
+        <x:v>221</x:v>
+      </x:c>
+      <x:c r="B4" s="31" t="s">
         <x:v>222</x:v>
-      </x:c>
-      <x:c r="B4" s="31" t="s">
-        <x:v>223</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="32" t="s">
-        <x:v>224</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="B5" s="33" t="str">
         <x:v>目标模型原生或系统级支持图、文、音频中的至少两种模态；具体攻击样本可为单模态或多模态，用于比较跨模态安全一致性。纯文本LLM、纯ASR、纯图像分类模型不纳入。</x:v>
@@ -12861,18 +13331,18 @@
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="32" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="B6" s="33" t="s">
         <x:v>225</x:v>
-      </x:c>
-      <x:c r="B6" s="33" t="s">
-        <x:v>226</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="32" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="B7" s="33" t="s">
         <x:v>227</x:v>
-      </x:c>
-      <x:c r="B7" s="33" t="s">
-        <x:v>228</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -12885,79 +13355,79 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="32" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="B9" s="33" t="s">
         <x:v>229</x:v>
-      </x:c>
-      <x:c r="B9" s="33" t="s">
-        <x:v>230</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="32" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="B10" s="33" t="s">
         <x:v>231</x:v>
-      </x:c>
-      <x:c r="B10" s="33" t="s">
-        <x:v>232</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="32" t="s">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="B11" s="33" t="s">
         <x:v>233</x:v>
-      </x:c>
-      <x:c r="B11" s="33" t="s">
-        <x:v>234</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="32" t="s">
+        <x:v>234</x:v>
+      </x:c>
+      <x:c r="B12" s="33" t="s">
         <x:v>235</x:v>
-      </x:c>
-      <x:c r="B12" s="33" t="s">
-        <x:v>236</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="32" t="s">
+        <x:v>236</x:v>
+      </x:c>
+      <x:c r="B13" s="33" t="s">
         <x:v>237</x:v>
-      </x:c>
-      <x:c r="B13" s="33" t="s">
-        <x:v>238</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="32" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="B14" s="33" t="s">
         <x:v>239</x:v>
-      </x:c>
-      <x:c r="B14" s="33" t="s">
-        <x:v>240</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="32" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="B15" s="33" t="s">
         <x:v>241</x:v>
-      </x:c>
-      <x:c r="B15" s="33" t="s">
-        <x:v>242</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="32" t="s">
+        <x:v>242</x:v>
+      </x:c>
+      <x:c r="B16" s="33" t="s">
         <x:v>243</x:v>
-      </x:c>
-      <x:c r="B16" s="33" t="s">
-        <x:v>244</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="32" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="B17" s="33" t="s">
         <x:v>245</x:v>
-      </x:c>
-      <x:c r="B17" s="33" t="s">
-        <x:v>246</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="32" t="s">
-        <x:v>247</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="B18" s="33" t="str">
         <x:v>不可感知扰动、分布式语义、跨模态重构、结构化输入异常或中间状态操控。</x:v>
@@ -12965,103 +13435,103 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="32" t="s">
+        <x:v>247</x:v>
+      </x:c>
+      <x:c r="B19" s="33" t="s">
         <x:v>248</x:v>
-      </x:c>
-      <x:c r="B19" s="33" t="s">
-        <x:v>249</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="32" t="s">
+        <x:v>249</x:v>
+      </x:c>
+      <x:c r="B20" s="33" t="s">
         <x:v>250</x:v>
-      </x:c>
-      <x:c r="B20" s="33" t="s">
-        <x:v>251</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="32" t="s">
+        <x:v>251</x:v>
+      </x:c>
+      <x:c r="B21" s="34" t="s">
         <x:v>252</x:v>
-      </x:c>
-      <x:c r="B21" s="34" t="s">
-        <x:v>253</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="32" t="s">
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="B22" s="33" t="s">
         <x:v>254</x:v>
-      </x:c>
-      <x:c r="B22" s="33" t="s">
-        <x:v>255</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A23" s="32" t="s">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="B23" s="33" t="s">
         <x:v>256</x:v>
-      </x:c>
-      <x:c r="B23" s="33" t="s">
-        <x:v>257</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="32" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="B24" s="33" t="s">
         <x:v>258</x:v>
-      </x:c>
-      <x:c r="B24" s="33" t="s">
-        <x:v>259</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A25" s="32" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="B25" s="33" t="s">
         <x:v>260</x:v>
-      </x:c>
-      <x:c r="B25" s="33" t="s">
-        <x:v>261</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="32" t="s">
+        <x:v>261</x:v>
+      </x:c>
+      <x:c r="B26" s="33" t="s">
         <x:v>262</x:v>
-      </x:c>
-      <x:c r="B26" s="33" t="s">
-        <x:v>263</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="32" t="s">
+        <x:v>263</x:v>
+      </x:c>
+      <x:c r="B27" s="33" t="s">
         <x:v>264</x:v>
-      </x:c>
-      <x:c r="B27" s="33" t="s">
-        <x:v>265</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="32" t="s">
+        <x:v>265</x:v>
+      </x:c>
+      <x:c r="B28" s="33" t="s">
         <x:v>266</x:v>
-      </x:c>
-      <x:c r="B28" s="33" t="s">
-        <x:v>267</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="32" t="s">
+        <x:v>267</x:v>
+      </x:c>
+      <x:c r="B29" s="33" t="s">
         <x:v>268</x:v>
-      </x:c>
-      <x:c r="B29" s="33" t="s">
-        <x:v>269</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="32" t="s">
+        <x:v>269</x:v>
+      </x:c>
+      <x:c r="B30" s="33" t="s">
         <x:v>270</x:v>
-      </x:c>
-      <x:c r="B30" s="33" t="s">
-        <x:v>271</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="32" t="s">
-        <x:v>272</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="B31" s="33" t="str">
         <x:v>来源与代码状态核验截至2026-08-26；论文指标受模型版本、评测集和判别器影响，不宜跨论文直接横比。</x:v>

</xml_diff>

<commit_message>
Refine taxonomy issue annotations
</commit_message>
<xml_diff>
--- a/面向多模态模型的攻击方法体系化梳理_2026-08-21_机制分类合并版.xlsx
+++ b/面向多模态模型的攻击方法体系化梳理_2026-08-21_机制分类合并版.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Re0d2368a12d6484c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类树" sheetId="2" r:id="R3e3a89fb698b4e51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="方法库" sheetId="3" r:id="R635a9fa01fe44330"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源清单" sheetId="4" r:id="R6d1c44e8e7844892"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径与评分" sheetId="5" r:id="R910d63f19dbf4b36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R826f74aff6fb4b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类树" sheetId="2" r:id="R4a760dbd535041e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="方法库" sheetId="3" r:id="R3b4deec55b0a4c77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源清单" sheetId="4" r:id="R61d039e2c8bf4d66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径与评分" sheetId="5" r:id="R40d035eaea4a42f1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4184,7 +4184,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7a26514555314587"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R787ad7c7c5534cb0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4194,19 +4194,6 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TaxonomyOldTable" displayName="TaxonomyOldTable" ref="A4:E24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="5">
-    <x:tableColumn id="1" name="一级分类"/>
-    <x:tableColumn id="2" name="二级分类（攻击原理）"/>
-    <x:tableColumn id="3" name="原理摘要"/>
-    <x:tableColumn id="4" name="代表方法"/>
-    <x:tableColumn id="5" name="该行存在的问题"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TaxonomyNewTable" displayName="TaxonomyNewTable" ref="A29:D47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="一级分类"/>
@@ -4215,6 +4202,18 @@
     <x:tableColumn id="4" name="代表方法"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TaxonomyOldTable" displayName="TaxonomyOldTable" ref="A4:D24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="一级分类"/>
+    <x:tableColumn id="2" name="二级分类（攻击原理）"/>
+    <x:tableColumn id="3" name="原理摘要"/>
+    <x:tableColumn id="4" name="代表方法"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -4693,7 +4692,7 @@
     <x:mergeCell ref="A27:H27"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ffa0bf72895468b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R371334ed6dd04121"/>
 </x:worksheet>
 </file>
 
@@ -4742,9 +4741,7 @@
       <x:c r="D4" s="131" t="str">
         <x:v>代表方法</x:v>
       </x:c>
-      <x:c r="E4" s="131" t="str">
-        <x:v>该行存在的问题</x:v>
-      </x:c>
+      <x:c r="E4" s="131" t="str"/>
     </x:row>
     <x:row r="5" ht="66" hidden="0" customHeight="1">
       <x:c r="A5" s="138" t="str">
@@ -4980,9 +4977,7 @@
       <x:c r="D18" s="43" t="str">
         <x:v>Extract-DM</x:v>
       </x:c>
-      <x:c r="E18" s="136" t="str">
-        <x:v>属于训练数据提取/样本恢复目标，不是越狱或提示注入；本版研究范围暂不纳入数据提取。</x:v>
-      </x:c>
+      <x:c r="E18" s="136"/>
     </x:row>
     <x:row r="19" ht="66" hidden="0" customHeight="1">
       <x:c r="A19" s="142" t="str">
@@ -4997,9 +4992,7 @@
       <x:c r="D19" s="43" t="str">
         <x:v>SecMI</x:v>
       </x:c>
-      <x:c r="E19" s="136" t="str">
-        <x:v>属于成员推断的数据隐私攻击，与当前仅保留的越狱/提示注入目标不同；本版暂不纳入。</x:v>
-      </x:c>
+      <x:c r="E19" s="136"/>
     </x:row>
     <x:row r="20" ht="66" hidden="0" customHeight="1">
       <x:c r="A20" s="142" t="str">
@@ -5014,9 +5007,7 @@
       <x:c r="D20" s="43" t="str">
         <x:v>VL-MIA</x:v>
       </x:c>
-      <x:c r="E20" s="136" t="str">
-        <x:v>属于跨模态成员推断/置信度攻击，仍是数据提取方向；本版暂不纳入。</x:v>
-      </x:c>
+      <x:c r="E20" s="136"/>
     </x:row>
     <x:row r="21" ht="66" hidden="0" customHeight="1">
       <x:c r="A21" s="142" t="str">
@@ -5031,9 +5022,7 @@
       <x:c r="D21" s="43" t="str">
         <x:v>VideoMIA</x:v>
       </x:c>
-      <x:c r="E21" s="136" t="str">
-        <x:v>同时属于视频专属与成员推断方向，超出当前图、文、音频及越狱/提示注入范围。</x:v>
-      </x:c>
+      <x:c r="E21" s="136"/>
     </x:row>
     <x:row r="22" ht="66" hidden="0" customHeight="1">
       <x:c r="A22" s="142" t="str">
@@ -5048,9 +5037,7 @@
       <x:c r="D22" s="43" t="str">
         <x:v>UMID</x:v>
       </x:c>
-      <x:c r="E22" s="136" t="str">
-        <x:v>属于潜变量反演与成员推断的数据隐私攻击；本版暂不纳入。</x:v>
-      </x:c>
+      <x:c r="E22" s="136"/>
     </x:row>
     <x:row r="23" ht="66" hidden="0" customHeight="1">
       <x:c r="A23" s="142" t="str">
@@ -5065,9 +5052,7 @@
       <x:c r="D23" s="43" t="str">
         <x:v>GPT-4V SPA</x:v>
       </x:c>
-      <x:c r="E23" s="136" t="str">
-        <x:v>攻击目标是系统提示/隐藏规则泄露，属于数据提取；不要与SASP“利用系统提示辅助自动搜索”混为同一主机制。</x:v>
-      </x:c>
+      <x:c r="E23" s="136"/>
     </x:row>
     <x:row r="24" ht="66" hidden="0" customHeight="1">
       <x:c r="A24" s="142" t="str">
@@ -5082,9 +5067,7 @@
       <x:c r="D24" s="43" t="str">
         <x:v>Image Hijacks—Leak Context</x:v>
       </x:c>
-      <x:c r="E24" s="136" t="str">
-        <x:v>攻击目标是上下文/提示泄露，属于数据提取效果；与Image Hijacks的行为控制机制应分开，本版暂不纳入。</x:v>
-      </x:c>
+      <x:c r="E24" s="136"/>
     </x:row>
     <x:row r="25" ht="18" customHeight="1"/>
     <x:row r="26" ht="18" customHeight="1"/>
@@ -5413,8 +5396,8 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4ce4eeb67594ddc"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R773e56646ef24015"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02c382726fc74c41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7691ad6efcaa407f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11967,7 +11950,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6f0422081194973"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7839fbeda62e4760"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13266,7 +13249,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e5b4ec526a0444a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbcac03b28c144d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>